<commit_message>
remove compiled Python cache files from __pycache__ directories and update Excel file
</commit_message>
<xml_diff>
--- a/Thoi_Khoa_Bieu_Truong_9_Lop.xlsx
+++ b/Thoi_Khoa_Bieu_Truong_9_Lop.xlsx
@@ -710,7 +710,7 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>HĐTN
+          <t>Tiếng Việt
 (Đỗ Hương (GVCN 1A))</t>
         </is>
       </c>
@@ -903,8 +903,8 @@
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-(Đỗ Hương (GVCN 1A))</t>
+          <t>Đạo đức
+(Phượng)</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
@@ -921,8 +921,8 @@
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>Tự nhiên &amp; Xã hội
-(Phượng)</t>
+          <t>Tiếng Việt
+(Chiên (GVCN 2B))</t>
         </is>
       </c>
       <c r="H9" s="10" t="inlineStr">
@@ -966,8 +966,8 @@
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-(Đỗ Hương (GVCN 1A))</t>
+          <t>Âm nhạc
+(Tươi (Âm nhạc))</t>
         </is>
       </c>
       <c r="E10" s="10" t="inlineStr">
@@ -984,8 +984,8 @@
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-(Chiên (GVCN 2B))</t>
+          <t>TC Toán
+(Lập)</t>
         </is>
       </c>
       <c r="H10" s="10" t="inlineStr">
@@ -1100,8 +1100,8 @@
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Âm nhạc
-(Tươi (Âm nhạc))</t>
+          <t>HĐTN
+(Đỗ Hương (GVCN 1A))</t>
         </is>
       </c>
       <c r="E12" s="13" t="inlineStr">
@@ -1289,8 +1289,8 @@
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
-          <t>GDTC
-(Phượng)</t>
+          <t>Tiếng Việt
+(Đỗ Hương (GVCN 1A))</t>
         </is>
       </c>
       <c r="E15" s="13" t="inlineStr">
@@ -1482,8 +1482,8 @@
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Đạo đức
-(Phượng)</t>
+          <t>Tiếng Việt
+(Đỗ Hương (GVCN 1A))</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
@@ -1500,8 +1500,8 @@
       </c>
       <c r="G18" s="13" t="inlineStr">
         <is>
-          <t>TC Toán
-(Lập)</t>
+          <t>Tự nhiên &amp; Xã hội
+(Phượng)</t>
         </is>
       </c>
       <c r="H18" s="13" t="inlineStr">
@@ -2069,8 +2069,8 @@
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
-          <t>Tiếng Việt
-(Đỗ Hương (GVCN 1A))</t>
+          <t>TC Toán
+(Phượng)</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
@@ -2388,7 +2388,7 @@
       </c>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>TC Toán
+          <t>GDTC
 (Phượng)</t>
         </is>
       </c>
@@ -3127,7 +3127,7 @@
       <c r="D6" s="10" t="inlineStr"/>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>1A - HĐTN</t>
+          <t>1A - Tiếng Việt</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
@@ -3321,11 +3321,7 @@
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr"/>
-      <c r="E9" s="10" t="inlineStr">
-        <is>
-          <t>1A - Tiếng Việt</t>
-        </is>
-      </c>
+      <c r="E9" s="10" t="inlineStr"/>
       <c r="F9" s="10" t="inlineStr">
         <is>
           <t>1B - Tiếng Việt</t>
@@ -3336,7 +3332,11 @@
           <t>2A - Tiếng Việt</t>
         </is>
       </c>
-      <c r="H9" s="10" t="inlineStr"/>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>2B - Tiếng Việt</t>
+        </is>
+      </c>
       <c r="I9" s="10" t="inlineStr">
         <is>
           <t>3A - TC Toán</t>
@@ -3356,7 +3356,7 @@
       <c r="M9" s="10" t="inlineStr"/>
       <c r="N9" s="10" t="inlineStr">
         <is>
-          <t>2B - Tự nhiên &amp; Xã hội</t>
+          <t>1A - Đạo đức</t>
         </is>
       </c>
       <c r="O9" s="10" t="inlineStr"/>
@@ -3385,22 +3385,14 @@
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr"/>
-      <c r="E10" s="10" t="inlineStr">
-        <is>
-          <t>1A - Tiếng Việt</t>
-        </is>
-      </c>
+      <c r="E10" s="10" t="inlineStr"/>
       <c r="F10" s="10" t="inlineStr"/>
       <c r="G10" s="10" t="inlineStr">
         <is>
           <t>2A - Tiếng Việt</t>
         </is>
       </c>
-      <c r="H10" s="10" t="inlineStr">
-        <is>
-          <t>2B - Tiếng Việt</t>
-        </is>
-      </c>
+      <c r="H10" s="10" t="inlineStr"/>
       <c r="I10" s="10" t="inlineStr">
         <is>
           <t>3A - TTCM</t>
@@ -3427,7 +3419,11 @@
           <t>1B - Tự nhiên &amp; Xã hội</t>
         </is>
       </c>
-      <c r="O10" s="10" t="inlineStr"/>
+      <c r="O10" s="10" t="inlineStr">
+        <is>
+          <t>2B - TC Toán</t>
+        </is>
+      </c>
       <c r="P10" s="10" t="inlineStr"/>
       <c r="Q10" s="10" t="inlineStr">
         <is>
@@ -3435,7 +3431,11 @@
         </is>
       </c>
       <c r="R10" s="10" t="inlineStr"/>
-      <c r="S10" s="10" t="inlineStr"/>
+      <c r="S10" s="10" t="inlineStr">
+        <is>
+          <t>1A - Âm nhạc</t>
+        </is>
+      </c>
       <c r="T10" s="10" t="inlineStr"/>
       <c r="U10" s="10" t="inlineStr"/>
       <c r="V10" s="10" t="inlineStr"/>
@@ -3521,7 +3521,11 @@
         </is>
       </c>
       <c r="D12" s="13" t="inlineStr"/>
-      <c r="E12" s="13" t="inlineStr"/>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>1A - HĐTN</t>
+        </is>
+      </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
           <t>1B - Toán</t>
@@ -3567,11 +3571,7 @@
           <t>4B - GDTC</t>
         </is>
       </c>
-      <c r="S12" s="13" t="inlineStr">
-        <is>
-          <t>1A - Âm nhạc</t>
-        </is>
-      </c>
+      <c r="S12" s="13" t="inlineStr"/>
       <c r="T12" s="13" t="inlineStr"/>
       <c r="U12" s="13" t="inlineStr"/>
       <c r="V12" s="13" t="inlineStr"/>
@@ -3713,7 +3713,11 @@
         </is>
       </c>
       <c r="D15" s="13" t="inlineStr"/>
-      <c r="E15" s="13" t="inlineStr"/>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>1A - Tiếng Việt</t>
+        </is>
+      </c>
       <c r="F15" s="13" t="inlineStr">
         <is>
           <t>1B - Tiếng Việt</t>
@@ -3746,11 +3750,7 @@
       </c>
       <c r="L15" s="13" t="inlineStr"/>
       <c r="M15" s="13" t="inlineStr"/>
-      <c r="N15" s="13" t="inlineStr">
-        <is>
-          <t>1A - GDTC</t>
-        </is>
-      </c>
+      <c r="N15" s="13" t="inlineStr"/>
       <c r="O15" s="13" t="inlineStr"/>
       <c r="P15" s="13" t="inlineStr"/>
       <c r="Q15" s="13" t="inlineStr"/>
@@ -3909,7 +3909,11 @@
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr"/>
-      <c r="E18" s="13" t="inlineStr"/>
+      <c r="E18" s="13" t="inlineStr">
+        <is>
+          <t>1A - Tiếng Việt</t>
+        </is>
+      </c>
       <c r="F18" s="13" t="inlineStr"/>
       <c r="G18" s="13" t="inlineStr">
         <is>
@@ -3936,14 +3940,10 @@
       <c r="M18" s="13" t="inlineStr"/>
       <c r="N18" s="13" t="inlineStr">
         <is>
-          <t>1A - Đạo đức</t>
-        </is>
-      </c>
-      <c r="O18" s="13" t="inlineStr">
-        <is>
-          <t>2B - TC Toán</t>
-        </is>
-      </c>
+          <t>2B - Tự nhiên &amp; Xã hội</t>
+        </is>
+      </c>
+      <c r="O18" s="13" t="inlineStr"/>
       <c r="P18" s="13" t="inlineStr"/>
       <c r="Q18" s="13" t="inlineStr">
         <is>
@@ -4505,11 +4505,7 @@
         </is>
       </c>
       <c r="D27" s="13" t="inlineStr"/>
-      <c r="E27" s="13" t="inlineStr">
-        <is>
-          <t>1A - Tiếng Việt</t>
-        </is>
-      </c>
+      <c r="E27" s="13" t="inlineStr"/>
       <c r="F27" s="13" t="inlineStr"/>
       <c r="G27" s="13" t="inlineStr">
         <is>
@@ -4530,7 +4526,11 @@
           <t>5B - Tiếng Việt</t>
         </is>
       </c>
-      <c r="N27" s="13" t="inlineStr"/>
+      <c r="N27" s="13" t="inlineStr">
+        <is>
+          <t>1A - TC Toán</t>
+        </is>
+      </c>
       <c r="O27" s="13" t="inlineStr">
         <is>
           <t>3A - TC Toán</t>
@@ -4864,7 +4864,7 @@
       <c r="M32" s="13" t="inlineStr"/>
       <c r="N32" s="13" t="inlineStr">
         <is>
-          <t>1A - TC Toán</t>
+          <t>1A - GDTC</t>
         </is>
       </c>
       <c r="O32" s="13" t="inlineStr"/>

</xml_diff>